<commit_message>
feat: update FE for 5-level difficulty system and English-only interface
Changes:
- Updated admin form to display 5 difficulty levels (🟢🟡🟠🔴⚫)
- Changed CSS grid layout for difficulty options (2 columns, mobile-first)
- Updated daily_challenge template to show all 5 difficulty levels
- Updated admin dashboard difficulty column with emoji display
- Updated Excel template generator for 5 difficulty levels (1-5)
- Added Help sheet to Excel template with full documentation
- Replaced Vietnamese placeholders with English in forms
- All 65 tests passing
</commit_message>
<xml_diff>
--- a/app/static/templates/questions_template.xlsx
+++ b/app/static/templates/questions_template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Help" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +43,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="000277BD"/>
         <bgColor rgb="000277BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+        <bgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,13 +70,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -592,10 +602,382 @@
     <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Select: finance, career, or business" type="list">
       <formula1>"finance,career,business"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Select: 1, 2, or 3" type="list">
-      <formula1>"1,2,3"</formula1>
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Select: 1 (Very Easy), 2 (Easy), 3 (Medium), 4 (Hard), or 5 (Very Hard)" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Valid Values</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>English title (max 200 chars)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Compound Interest Calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>title_vi</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Vietnamese title (fallback to English)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tính Lãi Kép</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>English question (Markdown + LaTeX)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>You have **10M VNĐ** at **6%/year**. After 3 years: $$FV = PV × (1+r)^n$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>question_vi</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Vietnamese question (Markdown + LaTeX)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Bạn có **10 triệu VNĐ**...</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>option_a</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Leave blank for free-text questions</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>16,105,100</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>option_b</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Leave blank for free-text questions</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>17,100,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>option_c</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Leave blank for free-text questions</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>18,205,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>option_d</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Leave blank for free-text questions</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>19,500,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>answer</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>a/b/c/d for MC, or exact text for free-text</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>explanation</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>English explanation (Markdown + LaTeX)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Using formula: $FV = 10M × (1.06)^3 = 11.91M$</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>explanation_vi</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Vietnamese explanation (Markdown + LaTeX)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Sử dụng công thức...</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>daily_challenge | mini_game | real_world</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>daily_challenge</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>sub_category</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Optional*</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>finance | career | business (*required for real_world)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>difficulty</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>1 (🟢 Very Easy) | 2 (🟡 Easy) | 3 (🟠 Medium) | 4 (🔴 Hard) | 5 (⚫ Very Hard)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>time_limit</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Seconds (for mini_game mode only)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>